<commit_message>
Add complete synthetic questionnaire evidence trial
</commit_message>
<xml_diff>
--- a/sample/evidence/A-03-scheduled-waste-consignment-fy2025.xlsx
+++ b/sample/evidence/A-03-scheduled-waste-consignment-fy2025.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -675,6 +675,52 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Waste balance</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Total waste generated 214.7 metric tonnes; diverted from disposal 138.2 metric tonnes; directed to disposal 76.5 metric tonnes</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Klang plant</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Scheduled waste by code</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Total hazardous scheduled waste generated 12.6 metric tonnes, identified by waste code: SW410 4.8, SW305 2.9, SW110 3.1, SW409 1.8</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Klang plant</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>